<commit_message>
feat: log-analyzer, excel-reporter 다중 파일 및 폴더 지원 추가
- readme 업데이트와 주석 추가 및 강화
</commit_message>
<xml_diff>
--- a/02.tools/01.log-analyzer/결과/bug_report_2026-06-17.xlsx
+++ b/02.tools/01.log-analyzer/결과/bug_report_2026-06-17.xlsx
@@ -10,6 +10,8 @@
     <sheet name="전체 로그" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="버그 리포트" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="통계 요약" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="변경 사항" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="중복 버그" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -75,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -84,6 +86,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -584,12 +587,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="39" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="39" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -605,6 +609,11 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>심각도</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>로그 내용</t>
         </is>
       </c>
@@ -622,22 +631,32 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
           <t>ERROR: 캐릭터 충돌 BUG-001 at 14:30:22</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>BUG-042</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>15:10:05</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>ERROR: 프레임 드랍 BUG-042 at 15:10:05</t>
         </is>
@@ -655,6 +674,11 @@
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>ERROR: 서버 응답 없음 BUG-007 at 16:00:11</t>
         </is>
@@ -691,32 +715,32 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>ERROR</t>
         </is>
       </c>
-      <c r="B2" s="6" t="n">
+      <c r="B2" s="7" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>WARNING</t>
         </is>
       </c>
-      <c r="B3" s="7" t="n">
+      <c r="B3" s="8" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-      <c r="B4" s="8" t="n">
+      <c r="B4" s="9" t="n">
         <v>3</v>
       </c>
     </row>
@@ -728,6 +752,102 @@
       </c>
       <c r="B5" s="1" t="n">
         <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>버그ID</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>🆕 신규</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>BUG-042</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>🆕 신규</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>BUG-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>🆕 신규</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>BUG-007</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>버그ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>발생 횟수</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: csv 한글 깨짐 수정 (utf-8을 utf-8-sig로 수정)
</commit_message>
<xml_diff>
--- a/02.tools/01.log-analyzer/결과/bug_report_2026-06-17.xlsx
+++ b/02.tools/01.log-analyzer/결과/bug_report_2026-06-17.xlsx
@@ -765,11 +765,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -781,42 +781,6 @@
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>버그ID</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>🆕 신규</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>BUG-042</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>🆕 신규</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>BUG-001</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>🆕 신규</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>BUG-007</t>
         </is>
       </c>
     </row>

</xml_diff>